<commit_message>
Latest generated outputs 2026-03-24
</commit_message>
<xml_diff>
--- a/generated/spreadsheet/development-relating-to-the-onshore-extraction-of-oil-and-gas-extraction-oil-gas.xlsx
+++ b/generated/spreadsheet/development-relating-to-the-onshore-extraction-of-oil-and-gas-extraction-oil-gas.xlsx
@@ -3196,13 +3196,13 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>Day type</t>
+          <t>Schedule days[]</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr"/>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>Day or type of day</t>
+          <t>List of days or day categories that a schedule entry applies to</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Latest generated outputs 2026-04-02
</commit_message>
<xml_diff>
--- a/generated/spreadsheet/development-relating-to-the-onshore-extraction-of-oil-and-gas-extraction-oil-gas.xlsx
+++ b/generated/spreadsheet/development-relating-to-the-onshore-extraction-of-oil-and-gas-extraction-oil-gas.xlsx
@@ -5134,7 +5134,7 @@
       </c>
       <c r="H147" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>datetime</t>
         </is>
       </c>
       <c r="I147" s="2" t="inlineStr">
@@ -5339,7 +5339,7 @@
       </c>
       <c r="H154" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>datetime</t>
         </is>
       </c>
       <c r="I154" s="2" t="inlineStr">

</xml_diff>